<commit_message>
Final PFMEA agent - Det scores are generic from excel
</commit_message>
<xml_diff>
--- a/pfmea_org.xlsx
+++ b/pfmea_org.xlsx
@@ -8,45 +8,47 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\IITM_MTech\Python Practice\pfmea_Agent_6_sep\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B234DA0-0392-4A93-8081-05FFB55BCC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD125B3-898C-494F-B5C2-C2F880384C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1770" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1770" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="5" r:id="rId1"/>
-    <sheet name="PFMEA" sheetId="1" r:id="rId2"/>
-    <sheet name="P-DET" sheetId="8" r:id="rId3"/>
-    <sheet name="P-OCC" sheetId="7" r:id="rId4"/>
-    <sheet name="P-SEV" sheetId="6" r:id="rId5"/>
-    <sheet name="Assumptions" sheetId="4" r:id="rId6"/>
+    <sheet name="Risk Classification Sheet" sheetId="10" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="5" r:id="rId2"/>
+    <sheet name="PFMEA" sheetId="1" r:id="rId3"/>
+    <sheet name="Agent Benefits" sheetId="9" r:id="rId4"/>
+    <sheet name="P-DET" sheetId="8" r:id="rId5"/>
+    <sheet name="P-OCC" sheetId="7" r:id="rId6"/>
+    <sheet name="P-SEV" sheetId="6" r:id="rId7"/>
+    <sheet name="Assumptions" sheetId="4" r:id="rId8"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId7"/>
-  </externalReferences>
   <definedNames>
-    <definedName name="CustCoC">'[1]Summary 1'!$R$41</definedName>
-    <definedName name="d" localSheetId="3">#REF!</definedName>
+    <definedName name="CustCoC">#REF!</definedName>
+    <definedName name="d" localSheetId="5">#REF!</definedName>
     <definedName name="d">#REF!</definedName>
-    <definedName name="data" localSheetId="3">#REF!</definedName>
+    <definedName name="data" localSheetId="5">#REF!</definedName>
     <definedName name="data">#REF!</definedName>
-    <definedName name="_xlnm.Database" localSheetId="3">#REF!</definedName>
+    <definedName name="_xlnm.Database" localSheetId="5">#REF!</definedName>
     <definedName name="_xlnm.Database">#REF!</definedName>
+    <definedName name="Det" localSheetId="0">#REF!</definedName>
     <definedName name="Det">Assumptions!$B$34:$B$43</definedName>
-    <definedName name="FF1_Programming" localSheetId="3">#REF!</definedName>
+    <definedName name="FF1_Programming" localSheetId="5">#REF!</definedName>
     <definedName name="FF1_Programming">#REF!</definedName>
     <definedName name="FF2_Programming">#REF!</definedName>
     <definedName name="Hello">#REF!</definedName>
     <definedName name="Hello1">#REF!</definedName>
-    <definedName name="NEI_FF1" localSheetId="3">#REF!</definedName>
+    <definedName name="NEI_FF1" localSheetId="5">#REF!</definedName>
     <definedName name="NEI_FF1">#REF!</definedName>
+    <definedName name="Occur" localSheetId="0">#REF!</definedName>
     <definedName name="Occur">Assumptions!$B$22:$B$31</definedName>
-    <definedName name="Overall" localSheetId="3">#REF!</definedName>
+    <definedName name="Overall" localSheetId="5">#REF!</definedName>
     <definedName name="Overall">#REF!</definedName>
     <definedName name="p">#REF!</definedName>
     <definedName name="Plage">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'P-DET'!$A$1:$I$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'P-OCC'!$A$1:$K$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'P-SEV'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'P-DET'!$A$1:$I$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'P-OCC'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'P-SEV'!$A$1:$H$15</definedName>
+    <definedName name="Sev" localSheetId="0">#REF!</definedName>
     <definedName name="Sev">Assumptions!$B$10:$B$19</definedName>
     <definedName name="ww">TRUE</definedName>
   </definedNames>
@@ -203,7 +205,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="304">
   <si>
     <t>Quality Tools</t>
   </si>
@@ -1328,12 +1330,99 @@
   <si>
     <t>DFMEA PFMEA Gap analysis check</t>
   </si>
+  <si>
+    <t>Severity: Irrelevant text</t>
+  </si>
+  <si>
+    <t>Current Process</t>
+  </si>
+  <si>
+    <t>S: Reduced performance</t>
+  </si>
+  <si>
+    <t>Severity Zone</t>
+  </si>
+  <si>
+    <t>Occurrence</t>
+  </si>
+  <si>
+    <t>PRIORITY LEVEL</t>
+  </si>
+  <si>
+    <t>Detection Zone</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Detectopm</t>
+  </si>
+  <si>
+    <t>Map the process step with failure mode</t>
+  </si>
+  <si>
+    <t>Map the failure mode with effect of failure(s)</t>
+  </si>
+  <si>
+    <t>Select the most severe effect of failure</t>
+  </si>
+  <si>
+    <t>Verify cause of failure</t>
+  </si>
+  <si>
+    <t>Verify prevention controls</t>
+  </si>
+  <si>
+    <t>Verify severity for different effect(s) of failure using AIAG standard</t>
+  </si>
+  <si>
+    <t>Verify detection for different detection contrls using AIAG standard</t>
+  </si>
+  <si>
+    <t>Verify Occurrence score using AIAG standard</t>
+  </si>
+  <si>
+    <t>Verify detection zone using Risk Classification Sheet</t>
+  </si>
+  <si>
+    <t>Verify severity zone Risk Classification Sheet</t>
+  </si>
+  <si>
+    <t>Verify Risk Priority using Risk Classification Sheet</t>
+  </si>
+  <si>
+    <t>Perform DFMEA PFMEA gap analysis</t>
+  </si>
+  <si>
+    <t>Verify detection scores for Significant and Critical dimensions</t>
+  </si>
+  <si>
+    <t>PFMEA Review steps</t>
+  </si>
+  <si>
+    <t>Manual verification</t>
+  </si>
+  <si>
+    <t>New Process</t>
+  </si>
+  <si>
+    <t>LLM verification</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Need Contextual information about part &amp; manufacturing process</t>
+  </si>
+  <si>
+    <t>Priority Level</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1561,8 +1650,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1659,8 +1761,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="28">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -1973,8 +2081,165 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1985,8 +2250,9 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="174">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2247,6 +2513,52 @@
     <xf numFmtId="0" fontId="21" fillId="5" borderId="26" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="28" xfId="7" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="7"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="33" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="33" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="34" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="35" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="12" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="12" borderId="33" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="12" borderId="34" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="32" xfId="7" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="3" xfId="7" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="36" xfId="7" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="37" xfId="7" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="33" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2355,6 +2667,45 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="15" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="16" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="28" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="32" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="37" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="38" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="34" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="35" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="32" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="29" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="30" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="31" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="19" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -2437,13 +2788,14 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="8">
     <cellStyle name="Hyperlink 2" xfId="6" xr:uid="{EB4FB036-C011-46F6-8E89-03487A1F22D0}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{5F93F98F-B3B1-416B-8D5B-1CC7DD77F1D8}"/>
     <cellStyle name="Normal 21" xfId="3" xr:uid="{115F5A8B-0F23-456F-B9B5-5EA3CB05C609}"/>
     <cellStyle name="Normal 23" xfId="2" xr:uid="{728DBA71-DD48-48C9-8ADA-912DF5AED142}"/>
     <cellStyle name="Normal 3" xfId="5" xr:uid="{33632A87-91A6-4606-84E2-D12604944703}"/>
+    <cellStyle name="Normal 4" xfId="7" xr:uid="{33474B2D-44C1-4C8D-B20F-53DBB697ADC9}"/>
     <cellStyle name="Normal_DFMEA Explainit" xfId="4" xr:uid="{67FB4E4C-C94C-4847-9E8A-255FBB86FDD7}"/>
   </cellStyles>
   <dxfs count="3">
@@ -2485,13 +2837,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>19</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>34637</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>327001</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>132656</xdr:rowOff>
@@ -2553,7 +2905,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>969466</xdr:colOff>
+      <xdr:colOff>742771</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -2742,49 +3094,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Summary 1"/>
-      <sheetName val="Changes"/>
-      <sheetName val="MBO_Changes"/>
-      <sheetName val="Summary"/>
-      <sheetName val="Input"/>
-      <sheetName val="Output"/>
-      <sheetName val="8-bin"/>
-      <sheetName val="P&amp;L"/>
-      <sheetName val="Forex Anal"/>
-      <sheetName val="Exch"/>
-      <sheetName val="Plant Data"/>
-      <sheetName val="OEM-Engr-Product Data"/>
-      <sheetName val="Index"/>
-      <sheetName val="Instructions"/>
-      <sheetName val="Deviation"/>
-      <sheetName val="Change Record"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3083,6 +3392,1024 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{936C86F0-93CE-4BBA-9F7E-B3324C9F82A1}">
+  <dimension ref="A1:S35"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="8.88671875" style="86"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" s="85"/>
+      <c r="B1" s="144" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1" s="145"/>
+      <c r="D1" s="145"/>
+      <c r="E1" s="145"/>
+      <c r="F1" s="145"/>
+      <c r="G1" s="145"/>
+      <c r="H1" s="145"/>
+      <c r="I1" s="145"/>
+      <c r="J1" s="145"/>
+      <c r="K1" s="145"/>
+      <c r="L1" s="146"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="87"/>
+      <c r="B2" s="88"/>
+      <c r="C2" s="88">
+        <v>1</v>
+      </c>
+      <c r="D2" s="88">
+        <v>2</v>
+      </c>
+      <c r="E2" s="88">
+        <v>3</v>
+      </c>
+      <c r="F2" s="88">
+        <v>4</v>
+      </c>
+      <c r="G2" s="88">
+        <v>5</v>
+      </c>
+      <c r="H2" s="88">
+        <v>6</v>
+      </c>
+      <c r="I2" s="88">
+        <v>7</v>
+      </c>
+      <c r="J2" s="88">
+        <v>8</v>
+      </c>
+      <c r="K2" s="88">
+        <v>9</v>
+      </c>
+      <c r="L2" s="89">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="143" t="s">
+        <v>279</v>
+      </c>
+      <c r="B3" s="94">
+        <v>10</v>
+      </c>
+      <c r="C3" s="90">
+        <v>3</v>
+      </c>
+      <c r="D3" s="101">
+        <v>1</v>
+      </c>
+      <c r="E3" s="101">
+        <v>1</v>
+      </c>
+      <c r="F3" s="101">
+        <v>1</v>
+      </c>
+      <c r="G3" s="101">
+        <v>1</v>
+      </c>
+      <c r="H3" s="101">
+        <v>1</v>
+      </c>
+      <c r="I3" s="101">
+        <v>1</v>
+      </c>
+      <c r="J3" s="101">
+        <v>1</v>
+      </c>
+      <c r="K3" s="101">
+        <v>1</v>
+      </c>
+      <c r="L3" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="143"/>
+      <c r="B4" s="94">
+        <v>9</v>
+      </c>
+      <c r="C4" s="90">
+        <v>3</v>
+      </c>
+      <c r="D4" s="101">
+        <v>1</v>
+      </c>
+      <c r="E4" s="101">
+        <v>1</v>
+      </c>
+      <c r="F4" s="101">
+        <v>1</v>
+      </c>
+      <c r="G4" s="101">
+        <v>1</v>
+      </c>
+      <c r="H4" s="101">
+        <v>1</v>
+      </c>
+      <c r="I4" s="101">
+        <v>1</v>
+      </c>
+      <c r="J4" s="101">
+        <v>1</v>
+      </c>
+      <c r="K4" s="101">
+        <v>1</v>
+      </c>
+      <c r="L4" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="143"/>
+      <c r="B5" s="94">
+        <v>8</v>
+      </c>
+      <c r="C5" s="90">
+        <v>3</v>
+      </c>
+      <c r="D5" s="90">
+        <v>2</v>
+      </c>
+      <c r="E5" s="101">
+        <v>1</v>
+      </c>
+      <c r="F5" s="101">
+        <v>1</v>
+      </c>
+      <c r="G5" s="101">
+        <v>1</v>
+      </c>
+      <c r="H5" s="101">
+        <v>1</v>
+      </c>
+      <c r="I5" s="101">
+        <v>1</v>
+      </c>
+      <c r="J5" s="101">
+        <v>1</v>
+      </c>
+      <c r="K5" s="101">
+        <v>1</v>
+      </c>
+      <c r="L5" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="143"/>
+      <c r="B6" s="94">
+        <v>7</v>
+      </c>
+      <c r="C6" s="90">
+        <v>3</v>
+      </c>
+      <c r="D6" s="90">
+        <v>2</v>
+      </c>
+      <c r="E6" s="90">
+        <v>2</v>
+      </c>
+      <c r="F6" s="90">
+        <v>2</v>
+      </c>
+      <c r="G6" s="101">
+        <v>1</v>
+      </c>
+      <c r="H6" s="101">
+        <v>1</v>
+      </c>
+      <c r="I6" s="101">
+        <v>1</v>
+      </c>
+      <c r="J6" s="101">
+        <v>1</v>
+      </c>
+      <c r="K6" s="101">
+        <v>1</v>
+      </c>
+      <c r="L6" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="143"/>
+      <c r="B7" s="94">
+        <v>6</v>
+      </c>
+      <c r="C7" s="90">
+        <v>3</v>
+      </c>
+      <c r="D7" s="90">
+        <v>2</v>
+      </c>
+      <c r="E7" s="90">
+        <v>2</v>
+      </c>
+      <c r="F7" s="90">
+        <v>2</v>
+      </c>
+      <c r="G7" s="101">
+        <v>1</v>
+      </c>
+      <c r="H7" s="101">
+        <v>1</v>
+      </c>
+      <c r="I7" s="101">
+        <v>1</v>
+      </c>
+      <c r="J7" s="101">
+        <v>1</v>
+      </c>
+      <c r="K7" s="101">
+        <v>1</v>
+      </c>
+      <c r="L7" s="102">
+        <v>1</v>
+      </c>
+      <c r="O7" s="134" t="s">
+        <v>280</v>
+      </c>
+      <c r="P7" s="135"/>
+      <c r="Q7" s="135"/>
+      <c r="R7" s="135"/>
+      <c r="S7" s="136"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" s="143"/>
+      <c r="B8" s="94">
+        <v>5</v>
+      </c>
+      <c r="C8" s="90">
+        <v>3</v>
+      </c>
+      <c r="D8" s="90">
+        <v>3</v>
+      </c>
+      <c r="E8" s="90">
+        <v>2</v>
+      </c>
+      <c r="F8" s="90">
+        <v>2</v>
+      </c>
+      <c r="G8" s="90">
+        <v>2</v>
+      </c>
+      <c r="H8" s="90">
+        <v>2</v>
+      </c>
+      <c r="I8" s="101">
+        <v>1</v>
+      </c>
+      <c r="J8" s="101">
+        <v>1</v>
+      </c>
+      <c r="K8" s="101">
+        <v>1</v>
+      </c>
+      <c r="L8" s="102">
+        <v>1</v>
+      </c>
+      <c r="O8" s="137" t="s">
+        <v>281</v>
+      </c>
+      <c r="P8" s="96">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="92">
+        <v>2</v>
+      </c>
+      <c r="R8" s="92">
+        <v>2</v>
+      </c>
+      <c r="S8" s="93">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" s="143"/>
+      <c r="B9" s="94">
+        <v>4</v>
+      </c>
+      <c r="C9" s="90">
+        <v>3</v>
+      </c>
+      <c r="D9" s="90">
+        <v>3</v>
+      </c>
+      <c r="E9" s="90">
+        <v>3</v>
+      </c>
+      <c r="F9" s="90">
+        <v>3</v>
+      </c>
+      <c r="G9" s="90">
+        <v>2</v>
+      </c>
+      <c r="H9" s="90">
+        <v>2</v>
+      </c>
+      <c r="I9" s="101">
+        <v>1</v>
+      </c>
+      <c r="J9" s="101">
+        <v>1</v>
+      </c>
+      <c r="K9" s="101">
+        <v>1</v>
+      </c>
+      <c r="L9" s="102">
+        <v>1</v>
+      </c>
+      <c r="O9" s="138"/>
+      <c r="P9" s="94">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="101">
+        <v>1</v>
+      </c>
+      <c r="R9" s="90">
+        <v>2</v>
+      </c>
+      <c r="S9" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" s="143"/>
+      <c r="B10" s="94">
+        <v>3</v>
+      </c>
+      <c r="C10" s="90">
+        <v>3</v>
+      </c>
+      <c r="D10" s="90">
+        <v>3</v>
+      </c>
+      <c r="E10" s="90">
+        <v>3</v>
+      </c>
+      <c r="F10" s="90">
+        <v>3</v>
+      </c>
+      <c r="G10" s="90">
+        <v>3</v>
+      </c>
+      <c r="H10" s="90">
+        <v>3</v>
+      </c>
+      <c r="I10" s="90">
+        <v>2</v>
+      </c>
+      <c r="J10" s="90">
+        <v>2</v>
+      </c>
+      <c r="K10" s="101">
+        <v>1</v>
+      </c>
+      <c r="L10" s="102">
+        <v>1</v>
+      </c>
+      <c r="O10" s="138"/>
+      <c r="P10" s="94">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="101">
+        <v>1</v>
+      </c>
+      <c r="R10" s="101">
+        <v>1</v>
+      </c>
+      <c r="S10" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" s="143"/>
+      <c r="B11" s="94">
+        <v>2</v>
+      </c>
+      <c r="C11" s="90">
+        <v>3</v>
+      </c>
+      <c r="D11" s="90">
+        <v>3</v>
+      </c>
+      <c r="E11" s="90">
+        <v>3</v>
+      </c>
+      <c r="F11" s="90">
+        <v>3</v>
+      </c>
+      <c r="G11" s="90">
+        <v>3</v>
+      </c>
+      <c r="H11" s="90">
+        <v>3</v>
+      </c>
+      <c r="I11" s="90">
+        <v>2</v>
+      </c>
+      <c r="J11" s="90">
+        <v>2</v>
+      </c>
+      <c r="K11" s="101">
+        <v>1</v>
+      </c>
+      <c r="L11" s="102">
+        <v>1</v>
+      </c>
+      <c r="O11" s="97"/>
+      <c r="P11" s="98"/>
+      <c r="Q11" s="94">
+        <v>1</v>
+      </c>
+      <c r="R11" s="94">
+        <v>2</v>
+      </c>
+      <c r="S11" s="95">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="143"/>
+      <c r="B12" s="94">
+        <v>1</v>
+      </c>
+      <c r="C12" s="90">
+        <v>3</v>
+      </c>
+      <c r="D12" s="90">
+        <v>3</v>
+      </c>
+      <c r="E12" s="90">
+        <v>3</v>
+      </c>
+      <c r="F12" s="90">
+        <v>3</v>
+      </c>
+      <c r="G12" s="90">
+        <v>3</v>
+      </c>
+      <c r="H12" s="90">
+        <v>3</v>
+      </c>
+      <c r="I12" s="90">
+        <v>3</v>
+      </c>
+      <c r="J12" s="90">
+        <v>3</v>
+      </c>
+      <c r="K12" s="90">
+        <v>3</v>
+      </c>
+      <c r="L12" s="91">
+        <v>3</v>
+      </c>
+      <c r="O12" s="99"/>
+      <c r="P12" s="100"/>
+      <c r="Q12" s="139" t="s">
+        <v>278</v>
+      </c>
+      <c r="R12" s="139"/>
+      <c r="S12" s="140"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13" s="97"/>
+      <c r="B13" s="98"/>
+      <c r="C13" s="94">
+        <v>1</v>
+      </c>
+      <c r="D13" s="94">
+        <v>2</v>
+      </c>
+      <c r="E13" s="94">
+        <v>3</v>
+      </c>
+      <c r="F13" s="94">
+        <v>4</v>
+      </c>
+      <c r="G13" s="94">
+        <v>5</v>
+      </c>
+      <c r="H13" s="94">
+        <v>6</v>
+      </c>
+      <c r="I13" s="94">
+        <v>7</v>
+      </c>
+      <c r="J13" s="94">
+        <v>8</v>
+      </c>
+      <c r="K13" s="94">
+        <v>9</v>
+      </c>
+      <c r="L13" s="95">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="99"/>
+      <c r="B14" s="100"/>
+      <c r="C14" s="139" t="s">
+        <v>282</v>
+      </c>
+      <c r="D14" s="139"/>
+      <c r="E14" s="139"/>
+      <c r="F14" s="139"/>
+      <c r="G14" s="139"/>
+      <c r="H14" s="139"/>
+      <c r="I14" s="139"/>
+      <c r="J14" s="139"/>
+      <c r="K14" s="139"/>
+      <c r="L14" s="140"/>
+    </row>
+    <row r="15" spans="1:19" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A16" s="85"/>
+      <c r="B16" s="141" t="s">
+        <v>281</v>
+      </c>
+      <c r="C16" s="141"/>
+      <c r="D16" s="141"/>
+      <c r="E16" s="141"/>
+      <c r="F16" s="141"/>
+      <c r="G16" s="141"/>
+      <c r="H16" s="141"/>
+      <c r="I16" s="141"/>
+      <c r="J16" s="141"/>
+      <c r="K16" s="141"/>
+      <c r="L16" s="142"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="87"/>
+      <c r="B17" s="88"/>
+      <c r="C17" s="88">
+        <v>1</v>
+      </c>
+      <c r="D17" s="88">
+        <v>2</v>
+      </c>
+      <c r="E17" s="88">
+        <v>3</v>
+      </c>
+      <c r="F17" s="88">
+        <v>4</v>
+      </c>
+      <c r="G17" s="88">
+        <v>5</v>
+      </c>
+      <c r="H17" s="88">
+        <v>6</v>
+      </c>
+      <c r="I17" s="88">
+        <v>7</v>
+      </c>
+      <c r="J17" s="88">
+        <v>8</v>
+      </c>
+      <c r="K17" s="88">
+        <v>9</v>
+      </c>
+      <c r="L17" s="89">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" s="143" t="s">
+        <v>283</v>
+      </c>
+      <c r="B18" s="94">
+        <v>10</v>
+      </c>
+      <c r="C18" s="90">
+        <v>3</v>
+      </c>
+      <c r="D18" s="90">
+        <v>2</v>
+      </c>
+      <c r="E18" s="101">
+        <v>1</v>
+      </c>
+      <c r="F18" s="101">
+        <v>1</v>
+      </c>
+      <c r="G18" s="101">
+        <v>1</v>
+      </c>
+      <c r="H18" s="101">
+        <v>1</v>
+      </c>
+      <c r="I18" s="101">
+        <v>1</v>
+      </c>
+      <c r="J18" s="101">
+        <v>1</v>
+      </c>
+      <c r="K18" s="101">
+        <v>1</v>
+      </c>
+      <c r="L18" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="143"/>
+      <c r="B19" s="94">
+        <v>9</v>
+      </c>
+      <c r="C19" s="90">
+        <v>3</v>
+      </c>
+      <c r="D19" s="90">
+        <v>2</v>
+      </c>
+      <c r="E19" s="101">
+        <v>1</v>
+      </c>
+      <c r="F19" s="101">
+        <v>1</v>
+      </c>
+      <c r="G19" s="101">
+        <v>1</v>
+      </c>
+      <c r="H19" s="101">
+        <v>1</v>
+      </c>
+      <c r="I19" s="101">
+        <v>1</v>
+      </c>
+      <c r="J19" s="101">
+        <v>1</v>
+      </c>
+      <c r="K19" s="101">
+        <v>1</v>
+      </c>
+      <c r="L19" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" s="143"/>
+      <c r="B20" s="94">
+        <v>8</v>
+      </c>
+      <c r="C20" s="90">
+        <v>3</v>
+      </c>
+      <c r="D20" s="90">
+        <v>2</v>
+      </c>
+      <c r="E20" s="90">
+        <v>2</v>
+      </c>
+      <c r="F20" s="90">
+        <v>2</v>
+      </c>
+      <c r="G20" s="90">
+        <v>2</v>
+      </c>
+      <c r="H20" s="90">
+        <v>2</v>
+      </c>
+      <c r="I20" s="101">
+        <v>1</v>
+      </c>
+      <c r="J20" s="101">
+        <v>1</v>
+      </c>
+      <c r="K20" s="101">
+        <v>1</v>
+      </c>
+      <c r="L20" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="143"/>
+      <c r="B21" s="94">
+        <v>7</v>
+      </c>
+      <c r="C21" s="90">
+        <v>3</v>
+      </c>
+      <c r="D21" s="90">
+        <v>3</v>
+      </c>
+      <c r="E21" s="90">
+        <v>3</v>
+      </c>
+      <c r="F21" s="90">
+        <v>2</v>
+      </c>
+      <c r="G21" s="90">
+        <v>2</v>
+      </c>
+      <c r="H21" s="90">
+        <v>2</v>
+      </c>
+      <c r="I21" s="90">
+        <v>2</v>
+      </c>
+      <c r="J21" s="101">
+        <v>1</v>
+      </c>
+      <c r="K21" s="101">
+        <v>1</v>
+      </c>
+      <c r="L21" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="143"/>
+      <c r="B22" s="94">
+        <v>6</v>
+      </c>
+      <c r="C22" s="90">
+        <v>3</v>
+      </c>
+      <c r="D22" s="90">
+        <v>3</v>
+      </c>
+      <c r="E22" s="90">
+        <v>3</v>
+      </c>
+      <c r="F22" s="90">
+        <v>3</v>
+      </c>
+      <c r="G22" s="90">
+        <v>3</v>
+      </c>
+      <c r="H22" s="90">
+        <v>2</v>
+      </c>
+      <c r="I22" s="90">
+        <v>2</v>
+      </c>
+      <c r="J22" s="101">
+        <v>1</v>
+      </c>
+      <c r="K22" s="101">
+        <v>1</v>
+      </c>
+      <c r="L22" s="102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="143"/>
+      <c r="B23" s="94">
+        <v>5</v>
+      </c>
+      <c r="C23" s="90">
+        <v>3</v>
+      </c>
+      <c r="D23" s="90">
+        <v>3</v>
+      </c>
+      <c r="E23" s="90">
+        <v>3</v>
+      </c>
+      <c r="F23" s="90">
+        <v>3</v>
+      </c>
+      <c r="G23" s="90">
+        <v>3</v>
+      </c>
+      <c r="H23" s="90">
+        <v>3</v>
+      </c>
+      <c r="I23" s="90">
+        <v>3</v>
+      </c>
+      <c r="J23" s="90">
+        <v>2</v>
+      </c>
+      <c r="K23" s="90">
+        <v>2</v>
+      </c>
+      <c r="L23" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" s="143"/>
+      <c r="B24" s="94">
+        <v>4</v>
+      </c>
+      <c r="C24" s="90">
+        <v>3</v>
+      </c>
+      <c r="D24" s="90">
+        <v>3</v>
+      </c>
+      <c r="E24" s="90">
+        <v>3</v>
+      </c>
+      <c r="F24" s="90">
+        <v>3</v>
+      </c>
+      <c r="G24" s="90">
+        <v>3</v>
+      </c>
+      <c r="H24" s="90">
+        <v>3</v>
+      </c>
+      <c r="I24" s="90">
+        <v>3</v>
+      </c>
+      <c r="J24" s="90">
+        <v>2</v>
+      </c>
+      <c r="K24" s="90">
+        <v>2</v>
+      </c>
+      <c r="L24" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" s="143"/>
+      <c r="B25" s="94">
+        <v>3</v>
+      </c>
+      <c r="C25" s="90">
+        <v>3</v>
+      </c>
+      <c r="D25" s="90">
+        <v>3</v>
+      </c>
+      <c r="E25" s="90">
+        <v>3</v>
+      </c>
+      <c r="F25" s="90">
+        <v>3</v>
+      </c>
+      <c r="G25" s="90">
+        <v>3</v>
+      </c>
+      <c r="H25" s="90">
+        <v>3</v>
+      </c>
+      <c r="I25" s="90">
+        <v>3</v>
+      </c>
+      <c r="J25" s="90">
+        <v>3</v>
+      </c>
+      <c r="K25" s="90">
+        <v>3</v>
+      </c>
+      <c r="L25" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="143"/>
+      <c r="B26" s="94">
+        <v>2</v>
+      </c>
+      <c r="C26" s="90">
+        <v>3</v>
+      </c>
+      <c r="D26" s="90">
+        <v>3</v>
+      </c>
+      <c r="E26" s="90">
+        <v>3</v>
+      </c>
+      <c r="F26" s="90">
+        <v>3</v>
+      </c>
+      <c r="G26" s="90">
+        <v>3</v>
+      </c>
+      <c r="H26" s="90">
+        <v>3</v>
+      </c>
+      <c r="I26" s="90">
+        <v>3</v>
+      </c>
+      <c r="J26" s="90">
+        <v>3</v>
+      </c>
+      <c r="K26" s="90">
+        <v>3</v>
+      </c>
+      <c r="L26" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="143"/>
+      <c r="B27" s="94">
+        <v>1</v>
+      </c>
+      <c r="C27" s="90">
+        <v>3</v>
+      </c>
+      <c r="D27" s="90">
+        <v>3</v>
+      </c>
+      <c r="E27" s="90">
+        <v>3</v>
+      </c>
+      <c r="F27" s="90">
+        <v>3</v>
+      </c>
+      <c r="G27" s="90">
+        <v>3</v>
+      </c>
+      <c r="H27" s="90">
+        <v>3</v>
+      </c>
+      <c r="I27" s="90">
+        <v>3</v>
+      </c>
+      <c r="J27" s="90">
+        <v>3</v>
+      </c>
+      <c r="K27" s="90">
+        <v>3</v>
+      </c>
+      <c r="L27" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="97"/>
+      <c r="B28" s="98"/>
+      <c r="C28" s="94">
+        <v>1</v>
+      </c>
+      <c r="D28" s="94">
+        <v>2</v>
+      </c>
+      <c r="E28" s="94">
+        <v>3</v>
+      </c>
+      <c r="F28" s="94">
+        <v>4</v>
+      </c>
+      <c r="G28" s="94">
+        <v>5</v>
+      </c>
+      <c r="H28" s="94">
+        <v>6</v>
+      </c>
+      <c r="I28" s="94">
+        <v>7</v>
+      </c>
+      <c r="J28" s="94">
+        <v>8</v>
+      </c>
+      <c r="K28" s="94">
+        <v>9</v>
+      </c>
+      <c r="L28" s="95">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="99"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="139" t="s">
+        <v>282</v>
+      </c>
+      <c r="D29" s="139"/>
+      <c r="E29" s="139"/>
+      <c r="F29" s="139"/>
+      <c r="G29" s="139"/>
+      <c r="H29" s="139"/>
+      <c r="I29" s="139"/>
+      <c r="J29" s="139"/>
+      <c r="K29" s="139"/>
+      <c r="L29" s="140"/>
+    </row>
+    <row r="33" ht="35.4" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="31.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="46.8" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A18:A27"/>
+    <mergeCell ref="C29:L29"/>
+    <mergeCell ref="B1:L1"/>
+    <mergeCell ref="A3:A12"/>
+    <mergeCell ref="O7:S7"/>
+    <mergeCell ref="O8:O10"/>
+    <mergeCell ref="Q12:S12"/>
+    <mergeCell ref="C14:L14"/>
+    <mergeCell ref="B16:L16"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E4E5BB-822F-4615-89D8-E2D73F4F0580}">
   <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3245,33 +4572,36 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:U23"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
     <col min="2" max="3" width="25.6640625" customWidth="1"/>
     <col min="4" max="4" width="3.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.88671875" customWidth="1"/>
+    <col min="5" max="5" width="3.6640625" customWidth="1"/>
     <col min="6" max="7" width="28.5546875" customWidth="1"/>
     <col min="8" max="8" width="5.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="9" max="9" width="23.33203125" customWidth="1"/>
     <col min="10" max="10" width="5.109375" customWidth="1"/>
     <col min="11" max="11" width="5.6640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16.5546875" customWidth="1"/>
-    <col min="13" max="13" width="15.5546875" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" style="1" customWidth="1"/>
-    <col min="15" max="17" width="3.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5" style="1" customWidth="1"/>
+    <col min="12" max="12" width="19.6640625" customWidth="1"/>
+    <col min="13" max="13" width="11.77734375" customWidth="1"/>
+    <col min="14" max="14" width="13.44140625" customWidth="1"/>
+    <col min="15" max="15" width="13.109375" customWidth="1"/>
+    <col min="16" max="16" width="15.5546875" customWidth="1"/>
+    <col min="17" max="17" width="12.6640625" style="1" customWidth="1"/>
+    <col min="18" max="20" width="3.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="30.6" x14ac:dyDescent="0.5">
-      <c r="A1" s="91" t="s">
+    <row r="1" spans="1:21" ht="30.6" x14ac:dyDescent="0.5">
+      <c r="A1" s="113" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="91"/>
-      <c r="C1" s="91"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
       <c r="F1" s="34" t="s">
@@ -3284,13 +4614,16 @@
       <c r="K1" s="18"/>
       <c r="L1" s="19"/>
       <c r="M1" s="19"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
       <c r="Q1" s="18"/>
       <c r="R1" s="18"/>
-    </row>
-    <row r="2" spans="1:18" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="S1" s="18"/>
+      <c r="T1" s="18"/>
+      <c r="U1" s="18"/>
+    </row>
+    <row r="2" spans="1:21" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A2" s="20" t="s">
         <v>66</v>
       </c>
@@ -3306,13 +4639,16 @@
       <c r="K2" s="18"/>
       <c r="L2" s="19"/>
       <c r="M2" s="19"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
       <c r="Q2" s="18"/>
       <c r="R2" s="18"/>
-    </row>
-    <row r="3" spans="1:18" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
+    </row>
+    <row r="3" spans="1:21" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
         <v>1</v>
       </c>
@@ -3330,213 +4666,237 @@
       <c r="K3" s="18"/>
       <c r="L3" s="19"/>
       <c r="M3" s="19"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
       <c r="Q3" s="18"/>
       <c r="R3" s="18"/>
-    </row>
-    <row r="4" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="100" t="s">
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
+    </row>
+    <row r="4" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="122" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="100"/>
-      <c r="C4" s="100"/>
+      <c r="B4" s="122"/>
+      <c r="C4" s="122"/>
       <c r="D4" s="18"/>
       <c r="E4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="92" t="s">
+      <c r="F4" s="114" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="92"/>
-      <c r="H4" s="92"/>
+      <c r="G4" s="114"/>
+      <c r="H4" s="114"/>
       <c r="I4" s="35"/>
       <c r="J4" s="24"/>
       <c r="K4" s="18"/>
-      <c r="L4" s="86" t="s">
+      <c r="L4" s="108" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="87"/>
-      <c r="N4" s="87"/>
-      <c r="O4" s="87"/>
-      <c r="P4" s="88"/>
-      <c r="Q4" s="90" t="s">
+      <c r="M4" s="109"/>
+      <c r="N4" s="109"/>
+      <c r="O4" s="109"/>
+      <c r="P4" s="109"/>
+      <c r="Q4" s="109"/>
+      <c r="R4" s="109"/>
+      <c r="S4" s="110"/>
+      <c r="T4" s="112" t="s">
         <v>27</v>
       </c>
-      <c r="R4" s="90"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="101"/>
-      <c r="B5" s="101"/>
-      <c r="C5" s="101"/>
+      <c r="U4" s="112"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A5" s="123"/>
+      <c r="B5" s="123"/>
+      <c r="C5" s="123"/>
       <c r="D5" s="25"/>
       <c r="E5" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="102" t="s">
+      <c r="F5" s="124" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="102"/>
-      <c r="H5" s="102"/>
+      <c r="G5" s="124"/>
+      <c r="H5" s="124"/>
       <c r="I5" s="35"/>
       <c r="J5" s="24"/>
       <c r="K5" s="25"/>
-      <c r="L5" s="86" t="s">
+      <c r="L5" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="M5" s="87"/>
-      <c r="N5" s="87"/>
-      <c r="O5" s="87"/>
-      <c r="P5" s="87"/>
-      <c r="Q5" s="88"/>
-      <c r="R5" s="26">
+      <c r="M5" s="109"/>
+      <c r="N5" s="109"/>
+      <c r="O5" s="109"/>
+      <c r="P5" s="109"/>
+      <c r="Q5" s="109"/>
+      <c r="R5" s="109"/>
+      <c r="S5" s="109"/>
+      <c r="T5" s="110"/>
+      <c r="U5" s="26">
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="101"/>
-      <c r="B6" s="101"/>
-      <c r="C6" s="101"/>
+    <row r="6" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="123"/>
+      <c r="B6" s="123"/>
+      <c r="C6" s="123"/>
       <c r="D6" s="25"/>
       <c r="E6" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="102" t="s">
+      <c r="F6" s="124" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="102"/>
-      <c r="H6" s="102"/>
+      <c r="G6" s="124"/>
+      <c r="H6" s="124"/>
       <c r="I6" s="35"/>
       <c r="J6" s="24"/>
       <c r="K6" s="18"/>
-      <c r="L6" s="86" t="s">
+      <c r="L6" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="M6" s="87"/>
-      <c r="N6" s="87"/>
-      <c r="O6" s="87"/>
-      <c r="P6" s="87"/>
-      <c r="Q6" s="88"/>
-      <c r="R6" s="26">
+      <c r="M6" s="109"/>
+      <c r="N6" s="109"/>
+      <c r="O6" s="109"/>
+      <c r="P6" s="109"/>
+      <c r="Q6" s="109"/>
+      <c r="R6" s="109"/>
+      <c r="S6" s="109"/>
+      <c r="T6" s="110"/>
+      <c r="U6" s="26">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="89" t="s">
+    <row r="7" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="111" t="s">
         <v>267</v>
       </c>
-      <c r="B7" s="89"/>
-      <c r="C7" s="89"/>
-      <c r="D7" s="89"/>
-      <c r="E7" s="89"/>
-      <c r="F7" s="89"/>
-      <c r="G7" s="89"/>
-      <c r="H7" s="89"/>
-      <c r="I7" s="89"/>
-      <c r="J7" s="89"/>
-      <c r="K7" s="89"/>
-      <c r="L7" s="89"/>
-      <c r="M7" s="89"/>
-      <c r="N7" s="89"/>
-      <c r="O7" s="89"/>
-      <c r="P7" s="89"/>
-      <c r="Q7" s="89"/>
-      <c r="R7" s="89"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B7" s="111"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="111"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="111"/>
+      <c r="I7" s="111"/>
+      <c r="J7" s="111"/>
+      <c r="K7" s="111"/>
+      <c r="L7" s="111"/>
+      <c r="M7" s="111"/>
+      <c r="N7" s="111"/>
+      <c r="O7" s="111"/>
+      <c r="P7" s="111"/>
+      <c r="Q7" s="111"/>
+      <c r="R7" s="111"/>
+      <c r="S7" s="111"/>
+      <c r="T7" s="111"/>
+      <c r="U7" s="111"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="98" t="s">
+      <c r="B8" s="120" t="s">
         <v>264</v>
       </c>
-      <c r="C8" s="98"/>
-      <c r="D8" s="98"/>
+      <c r="C8" s="120"/>
+      <c r="D8" s="120"/>
       <c r="E8" s="28"/>
-      <c r="F8" s="108" t="s">
+      <c r="F8" s="130" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="108"/>
-      <c r="H8" s="108"/>
-      <c r="I8" s="98" t="s">
+      <c r="G8" s="130"/>
+      <c r="H8" s="130"/>
+      <c r="I8" s="120" t="s">
         <v>269</v>
       </c>
-      <c r="J8" s="98"/>
-      <c r="K8" s="98"/>
+      <c r="J8" s="120"/>
+      <c r="K8" s="120"/>
       <c r="L8" s="28"/>
-      <c r="M8" s="27" t="s">
+      <c r="M8" s="28"/>
+      <c r="N8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="N8" s="98" t="s">
+      <c r="Q8" s="120" t="s">
         <v>65</v>
       </c>
-      <c r="O8" s="98"/>
-      <c r="P8" s="98"/>
-      <c r="Q8" s="98"/>
-      <c r="R8" s="98"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R8" s="120"/>
+      <c r="S8" s="120"/>
+      <c r="T8" s="120"/>
+      <c r="U8" s="120"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="98" t="s">
+      <c r="B9" s="120" t="s">
         <v>265</v>
       </c>
-      <c r="C9" s="98"/>
-      <c r="D9" s="98"/>
+      <c r="C9" s="120"/>
+      <c r="D9" s="120"/>
       <c r="E9" s="29"/>
-      <c r="F9" s="99" t="s">
+      <c r="F9" s="121" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="99"/>
-      <c r="H9" s="99"/>
-      <c r="I9" s="98" t="s">
+      <c r="G9" s="121"/>
+      <c r="H9" s="121"/>
+      <c r="I9" s="120" t="s">
         <v>268</v>
       </c>
-      <c r="J9" s="98"/>
-      <c r="K9" s="98"/>
+      <c r="J9" s="120"/>
+      <c r="K9" s="120"/>
       <c r="L9" s="28"/>
-      <c r="M9" s="27" t="s">
+      <c r="M9" s="28"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="N9" s="107"/>
-      <c r="O9" s="107"/>
-      <c r="P9" s="107"/>
-      <c r="Q9" s="107"/>
-      <c r="R9" s="107"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q9" s="129"/>
+      <c r="R9" s="129"/>
+      <c r="S9" s="129"/>
+      <c r="T9" s="129"/>
+      <c r="U9" s="129"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="103" t="s">
+      <c r="B10" s="125" t="s">
         <v>266</v>
       </c>
-      <c r="C10" s="103"/>
-      <c r="D10" s="103"/>
-      <c r="E10" s="103"/>
-      <c r="F10" s="103"/>
-      <c r="G10" s="103"/>
-      <c r="H10" s="103"/>
-      <c r="I10" s="103"/>
-      <c r="J10" s="103"/>
-      <c r="K10" s="103"/>
+      <c r="C10" s="125"/>
+      <c r="D10" s="125"/>
+      <c r="E10" s="125"/>
+      <c r="F10" s="125"/>
+      <c r="G10" s="125"/>
+      <c r="H10" s="125"/>
+      <c r="I10" s="125"/>
+      <c r="J10" s="125"/>
+      <c r="K10" s="125"/>
       <c r="L10" s="28"/>
-      <c r="M10" s="27" t="s">
+      <c r="M10" s="28"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="28"/>
+      <c r="P10" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="N10" s="30">
+      <c r="Q10" s="30">
         <v>46270</v>
       </c>
-      <c r="O10" s="109" t="s">
+      <c r="R10" s="131" t="s">
         <v>13</v>
       </c>
-      <c r="P10" s="109"/>
-      <c r="Q10" s="110"/>
-      <c r="R10" s="107"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S10" s="131"/>
+      <c r="T10" s="132"/>
+      <c r="U10" s="129"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="28"/>
       <c r="B11" s="28"/>
       <c r="C11" s="28"/>
@@ -3549,99 +4909,114 @@
       <c r="J11" s="28"/>
       <c r="K11" s="31"/>
       <c r="L11" s="28"/>
-      <c r="M11" s="27" t="s">
+      <c r="M11" s="28"/>
+      <c r="N11" s="28"/>
+      <c r="O11" s="28"/>
+      <c r="P11" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="N11" s="30">
+      <c r="Q11" s="30">
         <v>46270</v>
       </c>
-      <c r="O11" s="109" t="s">
+      <c r="R11" s="131" t="s">
         <v>13</v>
       </c>
-      <c r="P11" s="109"/>
-      <c r="Q11" s="110"/>
-      <c r="R11" s="107"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="93" t="s">
+      <c r="S11" s="131"/>
+      <c r="T11" s="132"/>
+      <c r="U11" s="129"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A12" s="115" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="85" t="s">
+      <c r="B12" s="107" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="85" t="s">
+      <c r="C12" s="107" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="95" t="s">
+      <c r="D12" s="117" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="96" t="s">
+      <c r="E12" s="118" t="s">
         <v>97</v>
       </c>
-      <c r="F12" s="85" t="s">
+      <c r="F12" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="G12" s="85" t="s">
+      <c r="G12" s="107" t="s">
         <v>234</v>
       </c>
-      <c r="H12" s="95" t="s">
+      <c r="H12" s="117" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="85" t="s">
+      <c r="I12" s="107" t="s">
         <v>235</v>
       </c>
-      <c r="J12" s="95" t="s">
+      <c r="J12" s="117" t="s">
         <v>25</v>
       </c>
-      <c r="K12" s="95" t="s">
+      <c r="K12" s="117" t="s">
         <v>19</v>
       </c>
-      <c r="L12" s="85" t="s">
+      <c r="L12" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="M12" s="85" t="s">
+      <c r="M12" s="107" t="s">
+        <v>278</v>
+      </c>
+      <c r="N12" s="107" t="s">
+        <v>281</v>
+      </c>
+      <c r="O12" s="107" t="s">
+        <v>303</v>
+      </c>
+      <c r="P12" s="107" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="111" t="s">
+      <c r="Q12" s="133" t="s">
         <v>22</v>
       </c>
-      <c r="O12" s="111"/>
-      <c r="P12" s="111"/>
-      <c r="Q12" s="111"/>
-      <c r="R12" s="111"/>
-    </row>
-    <row r="13" spans="1:18" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="94"/>
-      <c r="B13" s="85"/>
-      <c r="C13" s="85"/>
-      <c r="D13" s="95"/>
-      <c r="E13" s="97"/>
-      <c r="F13" s="85"/>
-      <c r="G13" s="85"/>
-      <c r="H13" s="95"/>
-      <c r="I13" s="85"/>
-      <c r="J13" s="95"/>
-      <c r="K13" s="95"/>
-      <c r="L13" s="85"/>
-      <c r="M13" s="85"/>
-      <c r="N13" s="32" t="s">
+      <c r="R12" s="133"/>
+      <c r="S12" s="133"/>
+      <c r="T12" s="133"/>
+      <c r="U12" s="133"/>
+    </row>
+    <row r="13" spans="1:21" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="116"/>
+      <c r="B13" s="107"/>
+      <c r="C13" s="107"/>
+      <c r="D13" s="117"/>
+      <c r="E13" s="119"/>
+      <c r="F13" s="107"/>
+      <c r="G13" s="107"/>
+      <c r="H13" s="117"/>
+      <c r="I13" s="107"/>
+      <c r="J13" s="117"/>
+      <c r="K13" s="117"/>
+      <c r="L13" s="107"/>
+      <c r="M13" s="107"/>
+      <c r="N13" s="107"/>
+      <c r="O13" s="107"/>
+      <c r="P13" s="107"/>
+      <c r="Q13" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="O13" s="33" t="s">
+      <c r="R13" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="P13" s="33" t="s">
+      <c r="S13" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="Q13" s="33" t="s">
+      <c r="T13" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="R13" s="33" t="s">
+      <c r="U13" s="33" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A14" s="104" t="s">
+    <row r="14" spans="1:21" ht="92.4" x14ac:dyDescent="0.25">
+      <c r="A14" s="126" t="s">
         <v>237</v>
       </c>
       <c r="B14" s="16" t="s">
@@ -3674,18 +5049,27 @@
         <v>28</v>
       </c>
       <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="14"/>
-      <c r="O14" s="14"/>
-      <c r="P14" s="14"/>
+      <c r="M14" s="13">
+        <v>2</v>
+      </c>
+      <c r="N14" s="13">
+        <v>1</v>
+      </c>
+      <c r="O14" s="13">
+        <v>2</v>
+      </c>
+      <c r="P14" s="13"/>
       <c r="Q14" s="14"/>
-      <c r="R14" s="2">
-        <f>IF(O14*P14*Q14&gt;0,O14*P14*Q14,K14)</f>
+      <c r="R14" s="14"/>
+      <c r="S14" s="14"/>
+      <c r="T14" s="14"/>
+      <c r="U14" s="2">
+        <f>IF(R14*S14*T14&gt;0,R14*S14*T14,K14)</f>
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A15" s="105"/>
+    <row r="15" spans="1:21" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A15" s="127"/>
       <c r="B15" s="13" t="s">
         <v>238</v>
       </c>
@@ -3718,18 +5102,27 @@
         <v>50</v>
       </c>
       <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="14"/>
-      <c r="P15" s="14"/>
+      <c r="M15" s="13">
+        <v>2</v>
+      </c>
+      <c r="N15" s="13">
+        <v>1</v>
+      </c>
+      <c r="O15" s="13">
+        <v>2</v>
+      </c>
+      <c r="P15" s="13"/>
       <c r="Q15" s="14"/>
-      <c r="R15" s="2">
-        <f t="shared" ref="R15:R23" si="1">IF(O15*P15*Q15&gt;0,O15*P15*Q15,K15)</f>
+      <c r="R15" s="14"/>
+      <c r="S15" s="14"/>
+      <c r="T15" s="14"/>
+      <c r="U15" s="2">
+        <f t="shared" ref="U15:U23" si="1">IF(R15*S15*T15&gt;0,R15*S15*T15,K15)</f>
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="118.8" x14ac:dyDescent="0.25">
-      <c r="A16" s="106"/>
+    <row r="16" spans="1:21" ht="118.8" x14ac:dyDescent="0.25">
+      <c r="A16" s="128"/>
       <c r="B16" s="15" t="s">
         <v>239</v>
       </c>
@@ -3760,17 +5153,26 @@
         <v>90</v>
       </c>
       <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="14"/>
+      <c r="M16" s="13">
+        <v>2</v>
+      </c>
+      <c r="N16" s="13">
+        <v>1</v>
+      </c>
+      <c r="O16" s="13">
+        <v>2</v>
+      </c>
+      <c r="P16" s="13"/>
       <c r="Q16" s="14"/>
-      <c r="R16" s="2">
+      <c r="R16" s="14"/>
+      <c r="S16" s="14"/>
+      <c r="T16" s="14"/>
+      <c r="U16" s="2">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="105.6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" ht="105.6" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13" t="s">
@@ -3800,17 +5202,26 @@
         <v>60</v>
       </c>
       <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="14"/>
-      <c r="P17" s="14"/>
+      <c r="M17" s="13">
+        <v>2</v>
+      </c>
+      <c r="N17" s="13">
+        <v>1</v>
+      </c>
+      <c r="O17" s="13">
+        <v>2</v>
+      </c>
+      <c r="P17" s="13"/>
       <c r="Q17" s="14"/>
-      <c r="R17" s="2">
+      <c r="R17" s="14"/>
+      <c r="S17" s="14"/>
+      <c r="T17" s="14"/>
+      <c r="U17" s="2">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="79.2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13" t="s">
@@ -3840,17 +5251,26 @@
         <v>64</v>
       </c>
       <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="14"/>
+      <c r="M18" s="13">
+        <v>2</v>
+      </c>
+      <c r="N18" s="13">
+        <v>1</v>
+      </c>
+      <c r="O18" s="13">
+        <v>2</v>
+      </c>
+      <c r="P18" s="13"/>
       <c r="Q18" s="14"/>
-      <c r="R18" s="2">
+      <c r="R18" s="14"/>
+      <c r="S18" s="14"/>
+      <c r="T18" s="14"/>
+      <c r="U18" s="2">
         <f t="shared" si="1"/>
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="105.6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" ht="105.6" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="15" t="s">
@@ -3880,17 +5300,26 @@
         <v>35</v>
       </c>
       <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="14"/>
-      <c r="O19" s="14"/>
-      <c r="P19" s="14"/>
+      <c r="M19" s="13">
+        <v>2</v>
+      </c>
+      <c r="N19" s="13">
+        <v>1</v>
+      </c>
+      <c r="O19" s="13">
+        <v>2</v>
+      </c>
+      <c r="P19" s="13"/>
       <c r="Q19" s="14"/>
-      <c r="R19" s="2">
+      <c r="R19" s="14"/>
+      <c r="S19" s="14"/>
+      <c r="T19" s="14"/>
+      <c r="U19" s="2">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="66" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13" t="s">
@@ -3920,28 +5349,37 @@
         <v>60</v>
       </c>
       <c r="L20" s="13"/>
-      <c r="M20" s="13"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="14"/>
+      <c r="M20" s="13">
+        <v>2</v>
+      </c>
+      <c r="N20" s="13">
+        <v>1</v>
+      </c>
+      <c r="O20" s="13">
+        <v>2</v>
+      </c>
+      <c r="P20" s="13"/>
       <c r="Q20" s="14"/>
-      <c r="R20" s="2">
+      <c r="R20" s="14"/>
+      <c r="S20" s="14"/>
+      <c r="T20" s="14"/>
+      <c r="U20" s="2">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="118.8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13" t="s">
-        <v>246</v>
+        <v>277</v>
       </c>
       <c r="D21" s="14">
         <v>9</v>
       </c>
       <c r="E21" s="13"/>
       <c r="F21" s="16" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>255</v>
@@ -3960,17 +5398,26 @@
         <v>216</v>
       </c>
       <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="14"/>
-      <c r="O21" s="14"/>
-      <c r="P21" s="14"/>
+      <c r="M21" s="13">
+        <v>2</v>
+      </c>
+      <c r="N21" s="13">
+        <v>1</v>
+      </c>
+      <c r="O21" s="13">
+        <v>2</v>
+      </c>
+      <c r="P21" s="13"/>
       <c r="Q21" s="14"/>
-      <c r="R21" s="2">
+      <c r="R21" s="14"/>
+      <c r="S21" s="14"/>
+      <c r="T21" s="14"/>
+      <c r="U21" s="2">
         <f t="shared" si="1"/>
         <v>216</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="118.8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" ht="118.8" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13" t="s">
@@ -4000,17 +5447,26 @@
         <v>504</v>
       </c>
       <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="14"/>
-      <c r="P22" s="14"/>
+      <c r="M22" s="13">
+        <v>2</v>
+      </c>
+      <c r="N22" s="13">
+        <v>1</v>
+      </c>
+      <c r="O22" s="13">
+        <v>2</v>
+      </c>
+      <c r="P22" s="13"/>
       <c r="Q22" s="14"/>
-      <c r="R22" s="2">
+      <c r="R22" s="14"/>
+      <c r="S22" s="14"/>
+      <c r="T22" s="14"/>
+      <c r="U22" s="2">
         <f t="shared" si="1"/>
         <v>504</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="92.4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" ht="92.4" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13" t="s">
@@ -4040,35 +5496,44 @@
         <v>84</v>
       </c>
       <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="14"/>
-      <c r="P23" s="14"/>
+      <c r="M23" s="13">
+        <v>2</v>
+      </c>
+      <c r="N23" s="13">
+        <v>1</v>
+      </c>
+      <c r="O23" s="13">
+        <v>2</v>
+      </c>
+      <c r="P23" s="13"/>
       <c r="Q23" s="14"/>
-      <c r="R23" s="2">
+      <c r="R23" s="14"/>
+      <c r="S23" s="14"/>
+      <c r="T23" s="14"/>
+      <c r="U23" s="2">
         <f t="shared" si="1"/>
         <v>84</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0"/>
-  <mergeCells count="38">
+  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0"/>
+  <mergeCells count="41">
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="N9:R9"/>
+    <mergeCell ref="Q9:U9"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="I8:K8"/>
-    <mergeCell ref="N8:R8"/>
+    <mergeCell ref="Q8:U8"/>
     <mergeCell ref="I9:K9"/>
     <mergeCell ref="K12:K13"/>
     <mergeCell ref="I12:I13"/>
     <mergeCell ref="L12:L13"/>
-    <mergeCell ref="O10:P10"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="M12:M13"/>
-    <mergeCell ref="N12:R12"/>
+    <mergeCell ref="R10:S10"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="R11:S11"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="P12:P13"/>
+    <mergeCell ref="Q12:U12"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="A12:A13"/>
@@ -4086,14 +5551,17 @@
     <mergeCell ref="F12:F13"/>
     <mergeCell ref="J12:J13"/>
     <mergeCell ref="G12:G13"/>
-    <mergeCell ref="L4:P4"/>
-    <mergeCell ref="L6:Q6"/>
-    <mergeCell ref="L5:Q5"/>
-    <mergeCell ref="A7:R7"/>
-    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="L4:S4"/>
+    <mergeCell ref="L6:T6"/>
+    <mergeCell ref="L5:T5"/>
+    <mergeCell ref="A7:U7"/>
+    <mergeCell ref="T4:U4"/>
+    <mergeCell ref="M12:M13"/>
+    <mergeCell ref="N12:N13"/>
+    <mergeCell ref="O12:O13"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="D14:D23 R14:R23">
+  <conditionalFormatting sqref="D14:D23 U14:U23">
     <cfRule type="cellIs" dxfId="2" priority="1" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
@@ -4103,19 +5571,19 @@
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O23">
+  <conditionalFormatting sqref="R14:R23">
     <cfRule type="cellIs" dxfId="0" priority="2" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O14:O23 D14:D23" xr:uid="{ADCE432E-9576-4B61-B09E-3538A1188765}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R14:R23 D14:D23" xr:uid="{ADCE432E-9576-4B61-B09E-3538A1188765}">
       <formula1>Sev</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H14:H23 P14:P23" xr:uid="{9448EF44-F384-4A47-BC1C-2D3E80CBC279}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H14:H23 S14:S23" xr:uid="{9448EF44-F384-4A47-BC1C-2D3E80CBC279}">
       <formula1>Occur</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J14:J23 Q14:Q23" xr:uid="{9736DCEB-4316-4210-AB5B-6E328600EF23}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J14:J23 T14:T23" xr:uid="{9736DCEB-4316-4210-AB5B-6E328600EF23}">
       <formula1>Det</formula1>
     </dataValidation>
   </dataValidations>
@@ -4126,7 +5594,204 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28C8645B-9559-4692-A29E-84C60693CCD6}">
+  <dimension ref="C2:F15"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="56.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C2" s="105" t="s">
+        <v>297</v>
+      </c>
+      <c r="D2" s="106" t="s">
+        <v>276</v>
+      </c>
+      <c r="E2" s="106" t="s">
+        <v>299</v>
+      </c>
+      <c r="F2" s="106" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="3" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C3" s="103" t="s">
+        <v>284</v>
+      </c>
+      <c r="D3" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E3" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="F3" s="103" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="4" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C4" s="103" t="s">
+        <v>285</v>
+      </c>
+      <c r="D4" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E4" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="F4" s="103" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="5" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C5" s="103" t="s">
+        <v>289</v>
+      </c>
+      <c r="D5" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E5" s="103" t="s">
+        <v>300</v>
+      </c>
+      <c r="F5" s="104"/>
+    </row>
+    <row r="6" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C6" s="103" t="s">
+        <v>286</v>
+      </c>
+      <c r="D6" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E6" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="F6" s="103" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C7" s="103" t="s">
+        <v>287</v>
+      </c>
+      <c r="D7" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E7" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="F7" s="103" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C8" s="103" t="s">
+        <v>288</v>
+      </c>
+      <c r="D8" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E8" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="F8" s="103" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C9" s="103" t="s">
+        <v>291</v>
+      </c>
+      <c r="D9" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E9" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="F9" s="103" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C10" s="103" t="s">
+        <v>290</v>
+      </c>
+      <c r="D10" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E10" s="103" t="s">
+        <v>300</v>
+      </c>
+      <c r="F10" s="104"/>
+    </row>
+    <row r="11" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C11" s="103" t="s">
+        <v>293</v>
+      </c>
+      <c r="D11" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E11" s="103" t="s">
+        <v>300</v>
+      </c>
+      <c r="F11" s="104"/>
+    </row>
+    <row r="12" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C12" s="103" t="s">
+        <v>292</v>
+      </c>
+      <c r="D12" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E12" s="103" t="s">
+        <v>300</v>
+      </c>
+      <c r="F12" s="104"/>
+    </row>
+    <row r="13" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C13" s="103" t="s">
+        <v>294</v>
+      </c>
+      <c r="D13" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E13" s="103" t="s">
+        <v>300</v>
+      </c>
+      <c r="F13" s="104"/>
+    </row>
+    <row r="14" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C14" s="103" t="s">
+        <v>295</v>
+      </c>
+      <c r="D14" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E14" s="103" t="s">
+        <v>300</v>
+      </c>
+      <c r="F14" s="104"/>
+    </row>
+    <row r="15" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C15" s="103" t="s">
+        <v>296</v>
+      </c>
+      <c r="D15" s="103" t="s">
+        <v>298</v>
+      </c>
+      <c r="E15" s="103" t="s">
+        <v>300</v>
+      </c>
+      <c r="F15" s="104"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28CEEFEA-4D67-49C3-9E22-C18C438E3D41}">
   <sheetPr>
     <tabColor rgb="FF99CCFF"/>
@@ -4152,35 +5817,35 @@
       </c>
     </row>
     <row r="2" spans="2:11" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="117" t="s">
+      <c r="B2" s="152" t="s">
         <v>204</v>
       </c>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="118"/>
-      <c r="H2" s="119"/>
+      <c r="C2" s="153"/>
+      <c r="D2" s="153"/>
+      <c r="E2" s="153"/>
+      <c r="F2" s="153"/>
+      <c r="G2" s="153"/>
+      <c r="H2" s="154"/>
       <c r="I2" s="74"/>
     </row>
     <row r="3" spans="2:11" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="42" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="120" t="s">
+      <c r="C3" s="155" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="121"/>
-      <c r="E3" s="122" t="s">
+      <c r="D3" s="156"/>
+      <c r="E3" s="157" t="s">
         <v>205</v>
       </c>
-      <c r="F3" s="122" t="s">
+      <c r="F3" s="157" t="s">
         <v>206</v>
       </c>
-      <c r="G3" s="122" t="s">
+      <c r="G3" s="157" t="s">
         <v>207</v>
       </c>
-      <c r="H3" s="124" t="s">
+      <c r="H3" s="159" t="s">
         <v>102</v>
       </c>
       <c r="I3" s="74"/>
@@ -4195,10 +5860,10 @@
       <c r="D4" s="43" t="s">
         <v>209</v>
       </c>
-      <c r="E4" s="123"/>
-      <c r="F4" s="123"/>
-      <c r="G4" s="123"/>
-      <c r="H4" s="124"/>
+      <c r="E4" s="158"/>
+      <c r="F4" s="158"/>
+      <c r="G4" s="158"/>
+      <c r="H4" s="159"/>
       <c r="K4" s="75"/>
     </row>
     <row r="5" spans="2:11" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4213,7 +5878,7 @@
       </c>
       <c r="E5" s="77"/>
       <c r="F5" s="78"/>
-      <c r="G5" s="112" t="s">
+      <c r="G5" s="147" t="s">
         <v>212</v>
       </c>
       <c r="H5" s="79"/>
@@ -4230,7 +5895,7 @@
       </c>
       <c r="E6" s="80"/>
       <c r="F6" s="78"/>
-      <c r="G6" s="113"/>
+      <c r="G6" s="148"/>
       <c r="H6" s="79"/>
     </row>
     <row r="7" spans="2:11" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4245,7 +5910,7 @@
       </c>
       <c r="E7" s="80"/>
       <c r="F7" s="78"/>
-      <c r="G7" s="113"/>
+      <c r="G7" s="148"/>
       <c r="H7" s="79"/>
     </row>
     <row r="8" spans="2:11" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4259,10 +5924,10 @@
         <v>218</v>
       </c>
       <c r="E8" s="80"/>
-      <c r="F8" s="112" t="s">
+      <c r="F8" s="147" t="s">
         <v>219</v>
       </c>
-      <c r="G8" s="113"/>
+      <c r="G8" s="148"/>
       <c r="H8" s="79"/>
     </row>
     <row r="9" spans="2:11" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4276,8 +5941,8 @@
         <v>220</v>
       </c>
       <c r="E9" s="80"/>
-      <c r="F9" s="114"/>
-      <c r="G9" s="113"/>
+      <c r="F9" s="149"/>
+      <c r="G9" s="148"/>
       <c r="H9" s="79"/>
     </row>
     <row r="10" spans="2:11" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4291,10 +5956,10 @@
         <v>221</v>
       </c>
       <c r="E10" s="80"/>
-      <c r="F10" s="112" t="s">
+      <c r="F10" s="147" t="s">
         <v>222</v>
       </c>
-      <c r="G10" s="114"/>
+      <c r="G10" s="149"/>
       <c r="H10" s="79"/>
     </row>
     <row r="11" spans="2:11" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4307,10 +5972,10 @@
       <c r="D11" s="76" t="s">
         <v>223</v>
       </c>
-      <c r="E11" s="112" t="s">
+      <c r="E11" s="147" t="s">
         <v>224</v>
       </c>
-      <c r="F11" s="113"/>
+      <c r="F11" s="148"/>
       <c r="G11" s="81"/>
       <c r="H11" s="79"/>
     </row>
@@ -4324,8 +5989,8 @@
       <c r="D12" s="76" t="s">
         <v>225</v>
       </c>
-      <c r="E12" s="115"/>
-      <c r="F12" s="114"/>
+      <c r="E12" s="150"/>
+      <c r="F12" s="149"/>
       <c r="G12" s="81"/>
       <c r="H12" s="79"/>
     </row>
@@ -4339,7 +6004,7 @@
       <c r="D13" s="76" t="s">
         <v>227</v>
       </c>
-      <c r="E13" s="115"/>
+      <c r="E13" s="150"/>
       <c r="F13" s="78"/>
       <c r="G13" s="81"/>
       <c r="H13" s="79"/>
@@ -4354,7 +6019,7 @@
       <c r="D14" s="76" t="s">
         <v>229</v>
       </c>
-      <c r="E14" s="116"/>
+      <c r="E14" s="151"/>
       <c r="F14" s="82"/>
       <c r="G14" s="83"/>
       <c r="H14" s="79"/>
@@ -4391,7 +6056,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B632E708-D59C-42F1-B1F6-CD8F4E41DE9D}">
   <sheetPr>
     <tabColor rgb="FF99CCFF"/>
@@ -4420,17 +6085,17 @@
       </c>
     </row>
     <row r="2" spans="2:11" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="117" t="s">
+      <c r="B2" s="152" t="s">
         <v>138</v>
       </c>
-      <c r="C2" s="125"/>
-      <c r="D2" s="125"/>
-      <c r="E2" s="125"/>
-      <c r="F2" s="125"/>
-      <c r="G2" s="125"/>
-      <c r="H2" s="125"/>
-      <c r="I2" s="125"/>
-      <c r="J2" s="126"/>
+      <c r="C2" s="160"/>
+      <c r="D2" s="160"/>
+      <c r="E2" s="160"/>
+      <c r="F2" s="160"/>
+      <c r="G2" s="160"/>
+      <c r="H2" s="160"/>
+      <c r="I2" s="160"/>
+      <c r="J2" s="161"/>
     </row>
     <row r="3" spans="2:11" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="42" t="s">
@@ -4439,65 +6104,65 @@
       <c r="C3" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="D3" s="120" t="s">
+      <c r="D3" s="155" t="s">
         <v>140</v>
       </c>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="121"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="156"/>
       <c r="H3" s="42" t="s">
         <v>141</v>
       </c>
       <c r="I3" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="J3" s="122" t="s">
+      <c r="J3" s="157" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="4" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="122" t="s">
+      <c r="B4" s="157" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="122" t="s">
+      <c r="C4" s="157" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="129" t="s">
+      <c r="D4" s="164" t="s">
         <v>144</v>
       </c>
-      <c r="E4" s="130"/>
-      <c r="F4" s="122" t="s">
+      <c r="E4" s="165"/>
+      <c r="F4" s="157" t="s">
         <v>145</v>
       </c>
-      <c r="G4" s="122" t="s">
+      <c r="G4" s="157" t="s">
         <v>146</v>
       </c>
-      <c r="H4" s="129" t="s">
+      <c r="H4" s="164" t="s">
         <v>147</v>
       </c>
-      <c r="I4" s="130"/>
-      <c r="J4" s="128" t="s">
+      <c r="I4" s="165"/>
+      <c r="J4" s="163" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="123"/>
-      <c r="C5" s="123"/>
+      <c r="B5" s="158"/>
+      <c r="C5" s="158"/>
       <c r="D5" s="43" t="s">
         <v>148</v>
       </c>
       <c r="E5" s="43" t="s">
         <v>146</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="123"/>
+      <c r="F5" s="158"/>
+      <c r="G5" s="158"/>
       <c r="H5" s="43" t="s">
         <v>148</v>
       </c>
       <c r="I5" s="43" t="s">
         <v>149</v>
       </c>
-      <c r="J5" s="123"/>
+      <c r="J5" s="158"/>
     </row>
     <row r="6" spans="2:11" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="45">
@@ -4530,7 +6195,7 @@
       <c r="B7" s="47">
         <v>9</v>
       </c>
-      <c r="C7" s="131" t="s">
+      <c r="C7" s="166" t="s">
         <v>156</v>
       </c>
       <c r="D7" s="61" t="s">
@@ -4557,7 +6222,7 @@
       <c r="B8" s="48">
         <v>8</v>
       </c>
-      <c r="C8" s="131"/>
+      <c r="C8" s="166"/>
       <c r="D8" s="61" t="s">
         <v>162</v>
       </c>
@@ -4582,7 +6247,7 @@
       <c r="B9" s="49">
         <v>7</v>
       </c>
-      <c r="C9" s="131"/>
+      <c r="C9" s="166"/>
       <c r="D9" s="61" t="s">
         <v>166</v>
       </c>
@@ -4607,7 +6272,7 @@
       <c r="B10" s="50">
         <v>6</v>
       </c>
-      <c r="C10" s="131" t="s">
+      <c r="C10" s="166" t="s">
         <v>171</v>
       </c>
       <c r="D10" s="61" t="s">
@@ -4634,7 +6299,7 @@
       <c r="B11" s="51">
         <v>5</v>
       </c>
-      <c r="C11" s="131"/>
+      <c r="C11" s="166"/>
       <c r="D11" s="61" t="s">
         <v>177</v>
       </c>
@@ -4659,7 +6324,7 @@
       <c r="B12" s="52">
         <v>4</v>
       </c>
-      <c r="C12" s="131"/>
+      <c r="C12" s="166"/>
       <c r="D12" s="61" t="s">
         <v>182</v>
       </c>
@@ -4684,7 +6349,7 @@
       <c r="B13" s="53">
         <v>3</v>
       </c>
-      <c r="C13" s="131" t="s">
+      <c r="C13" s="166" t="s">
         <v>187</v>
       </c>
       <c r="D13" s="61" t="s">
@@ -4711,7 +6376,7 @@
       <c r="B14" s="54">
         <v>2</v>
       </c>
-      <c r="C14" s="131"/>
+      <c r="C14" s="166"/>
       <c r="D14" s="61" t="s">
         <v>193</v>
       </c>
@@ -4775,14 +6440,14 @@
       </c>
     </row>
     <row r="17" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="132"/>
-      <c r="C17" s="132"/>
-      <c r="D17" s="132"/>
-      <c r="E17" s="132"/>
-      <c r="F17" s="132"/>
-      <c r="G17" s="132"/>
-      <c r="H17" s="132"/>
-      <c r="I17" s="132"/>
+      <c r="B17" s="167"/>
+      <c r="C17" s="167"/>
+      <c r="D17" s="167"/>
+      <c r="E17" s="167"/>
+      <c r="F17" s="167"/>
+      <c r="G17" s="167"/>
+      <c r="H17" s="167"/>
+      <c r="I17" s="167"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="70"/>
@@ -4798,15 +6463,15 @@
       <c r="B20" s="71"/>
       <c r="C20" s="71"/>
       <c r="D20" s="72"/>
-      <c r="H20" s="133"/>
-      <c r="I20" s="133"/>
+      <c r="H20" s="168"/>
+      <c r="I20" s="168"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="71"/>
       <c r="C21" s="71"/>
       <c r="D21" s="72"/>
-      <c r="H21" s="133"/>
-      <c r="I21" s="133"/>
+      <c r="H21" s="168"/>
+      <c r="I21" s="168"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -4843,7 +6508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA395079-6C96-4192-A492-E3C5F37226AD}">
   <sheetPr>
     <tabColor rgb="FF99CCFF"/>
@@ -4869,26 +6534,26 @@
       </c>
     </row>
     <row r="2" spans="2:8" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="117" t="s">
+      <c r="B2" s="152" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="125"/>
-      <c r="D2" s="125"/>
-      <c r="E2" s="125"/>
-      <c r="F2" s="125"/>
-      <c r="G2" s="126"/>
+      <c r="C2" s="160"/>
+      <c r="D2" s="160"/>
+      <c r="E2" s="160"/>
+      <c r="F2" s="160"/>
+      <c r="G2" s="161"/>
     </row>
     <row r="3" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="42" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="134" t="s">
+      <c r="C3" s="169" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="134"/>
-      <c r="E3" s="134"/>
-      <c r="F3" s="134"/>
-      <c r="G3" s="124" t="s">
+      <c r="D3" s="169"/>
+      <c r="E3" s="169"/>
+      <c r="F3" s="169"/>
+      <c r="G3" s="159" t="s">
         <v>102</v>
       </c>
     </row>
@@ -4908,10 +6573,10 @@
       <c r="F4" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="G4" s="124"/>
+      <c r="G4" s="159"/>
     </row>
     <row r="5" spans="2:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="131" t="s">
+      <c r="B5" s="166" t="s">
         <v>108</v>
       </c>
       <c r="C5" s="44" t="s">
@@ -4920,7 +6585,7 @@
       <c r="D5" s="45">
         <v>10</v>
       </c>
-      <c r="E5" s="131" t="s">
+      <c r="E5" s="166" t="s">
         <v>108</v>
       </c>
       <c r="F5" s="44" t="s">
@@ -4929,21 +6594,21 @@
       <c r="G5" s="46"/>
     </row>
     <row r="6" spans="2:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="131"/>
+      <c r="B6" s="166"/>
       <c r="C6" s="44" t="s">
         <v>111</v>
       </c>
       <c r="D6" s="47">
         <v>9</v>
       </c>
-      <c r="E6" s="131"/>
+      <c r="E6" s="166"/>
       <c r="F6" s="44" t="s">
         <v>112</v>
       </c>
       <c r="G6" s="46"/>
     </row>
     <row r="7" spans="2:8" ht="57.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="131" t="s">
+      <c r="B7" s="166" t="s">
         <v>113</v>
       </c>
       <c r="C7" s="44" t="s">
@@ -4961,7 +6626,7 @@
       <c r="G7" s="46"/>
     </row>
     <row r="8" spans="2:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="131"/>
+      <c r="B8" s="166"/>
       <c r="C8" s="44" t="s">
         <v>117</v>
       </c>
@@ -4977,7 +6642,7 @@
       <c r="G8" s="46"/>
     </row>
     <row r="9" spans="2:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="131" t="s">
+      <c r="B9" s="166" t="s">
         <v>120</v>
       </c>
       <c r="C9" s="44" t="s">
@@ -4986,7 +6651,7 @@
       <c r="D9" s="50">
         <v>6</v>
       </c>
-      <c r="E9" s="131" t="s">
+      <c r="E9" s="166" t="s">
         <v>122</v>
       </c>
       <c r="F9" s="44" t="s">
@@ -4995,21 +6660,21 @@
       <c r="G9" s="46"/>
     </row>
     <row r="10" spans="2:8" ht="55.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="131"/>
+      <c r="B10" s="166"/>
       <c r="C10" s="44" t="s">
         <v>124</v>
       </c>
       <c r="D10" s="51">
         <v>5</v>
       </c>
-      <c r="E10" s="131"/>
+      <c r="E10" s="166"/>
       <c r="F10" s="44" t="s">
         <v>125</v>
       </c>
       <c r="G10" s="46"/>
     </row>
     <row r="11" spans="2:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="131" t="s">
+      <c r="B11" s="166" t="s">
         <v>126</v>
       </c>
       <c r="C11" s="44" t="s">
@@ -5018,7 +6683,7 @@
       <c r="D11" s="52">
         <v>4</v>
       </c>
-      <c r="E11" s="131" t="s">
+      <c r="E11" s="166" t="s">
         <v>122</v>
       </c>
       <c r="F11" s="44" t="s">
@@ -5027,21 +6692,21 @@
       <c r="G11" s="46"/>
     </row>
     <row r="12" spans="2:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="131"/>
+      <c r="B12" s="166"/>
       <c r="C12" s="44" t="s">
         <v>129</v>
       </c>
       <c r="D12" s="53">
         <v>3</v>
       </c>
-      <c r="E12" s="131"/>
+      <c r="E12" s="166"/>
       <c r="F12" s="44" t="s">
         <v>130</v>
       </c>
       <c r="G12" s="46"/>
     </row>
     <row r="13" spans="2:8" ht="42" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="131"/>
+      <c r="B13" s="166"/>
       <c r="C13" s="44" t="s">
         <v>131</v>
       </c>
@@ -5109,7 +6774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C44"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -5132,34 +6797,34 @@
       <c r="B2" s="9"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="137" t="s">
+      <c r="A3" s="172" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="138"/>
+      <c r="B3" s="173"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="137" t="s">
+      <c r="A4" s="172" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="138"/>
+      <c r="B4" s="173"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="137" t="s">
+      <c r="A5" s="172" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="138"/>
+      <c r="B5" s="173"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="137" t="s">
+      <c r="A6" s="172" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="138"/>
+      <c r="B6" s="173"/>
     </row>
     <row r="7" spans="1:3" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="135" t="s">
+      <c r="A7" s="170" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="136"/>
+      <c r="B7" s="171"/>
     </row>
     <row r="8" spans="1:3" ht="14.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>

</xml_diff>